<commit_message>
clean notebook and update SAAM analysis
</commit_message>
<xml_diff>
--- a/notebooks/monthly_portfolio_returns_2014_2025.xlsx
+++ b/notebooks/monthly_portfolio_returns_2014_2025.xlsx
@@ -443,7 +443,7 @@
         <v>-0.03494855159817797</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.01037199718703215</v>
+        <v>-0.03494855159817797</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,7 @@
         <v>0.05470324098031322</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0337783544573695</v>
+        <v>0.05470324098031322</v>
       </c>
     </row>
     <row r="4">
@@ -469,7 +469,7 @@
         <v>0.009290254635864935</v>
       </c>
       <c r="C4" t="n">
-        <v>0.001343125713222268</v>
+        <v>0.009290254635864935</v>
       </c>
     </row>
     <row r="5">
@@ -482,7 +482,7 @@
         <v>0.01705414331523906</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01137885728269963</v>
+        <v>0.01705414331523906</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
         <v>0.01573781668140689</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01977176483312058</v>
+        <v>0.01573781668140689</v>
       </c>
     </row>
     <row r="7">
@@ -508,7 +508,7 @@
         <v>0.0135843254131045</v>
       </c>
       <c r="C7" t="n">
-        <v>0.03205882436507544</v>
+        <v>0.0135843254131045</v>
       </c>
     </row>
     <row r="8">
@@ -521,7 +521,7 @@
         <v>-0.02297284055523763</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.01306264743903388</v>
+        <v>-0.02297284055523763</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         <v>0.02728537359108229</v>
       </c>
       <c r="C9" t="n">
-        <v>0.03385130181039037</v>
+        <v>0.02728537359108229</v>
       </c>
     </row>
     <row r="10">
@@ -547,7 +547,7 @@
         <v>-0.02335601002647316</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.01689255327892198</v>
+        <v>-0.02335601002647316</v>
       </c>
     </row>
     <row r="11">
@@ -560,7 +560,7 @@
         <v>0.004632013532543199</v>
       </c>
       <c r="C11" t="n">
-        <v>0.04089385058689901</v>
+        <v>0.004632013532543199</v>
       </c>
     </row>
     <row r="12">
@@ -573,7 +573,7 @@
         <v>0.03041181054854081</v>
       </c>
       <c r="C12" t="n">
-        <v>0.02732133742957922</v>
+        <v>0.03041181054854081</v>
       </c>
     </row>
     <row r="13">
@@ -586,7 +586,7 @@
         <v>-0.01909033912522776</v>
       </c>
       <c r="C13" t="n">
-        <v>0.004260826341084613</v>
+        <v>-0.01909033912522776</v>
       </c>
     </row>
     <row r="14">
@@ -599,7 +599,7 @@
         <v>-0.01938885162887482</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.006380862069732324</v>
+        <v>-0.01938885162887482</v>
       </c>
     </row>
     <row r="15">
@@ -612,7 +612,7 @@
         <v>0.05742801269246856</v>
       </c>
       <c r="C15" t="n">
-        <v>0.03607735048066851</v>
+        <v>0.05742801269246856</v>
       </c>
     </row>
     <row r="16">
@@ -625,7 +625,7 @@
         <v>-0.01823988426294667</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.008906609926551939</v>
+        <v>-0.01823988426294667</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         <v>0.02302326507590106</v>
       </c>
       <c r="C17" t="n">
-        <v>0.01107304518116488</v>
+        <v>0.02302326507590106</v>
       </c>
     </row>
     <row r="18">
@@ -651,7 +651,7 @@
         <v>0.001559662658366811</v>
       </c>
       <c r="C18" t="n">
-        <v>0.01998017594918212</v>
+        <v>0.001559662658366811</v>
       </c>
     </row>
     <row r="19">
@@ -664,7 +664,7 @@
         <v>-0.02756496175961278</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.01138130075353012</v>
+        <v>-0.02756496175961278</v>
       </c>
     </row>
     <row r="20">
@@ -677,7 +677,7 @@
         <v>0.02337215247765667</v>
       </c>
       <c r="C20" t="n">
-        <v>0.02684300514003121</v>
+        <v>0.02337215247765667</v>
       </c>
     </row>
     <row r="21">
@@ -690,7 +690,7 @@
         <v>-0.0622245390646549</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.05461963195002752</v>
+        <v>-0.0622245390646549</v>
       </c>
     </row>
     <row r="22">
@@ -703,7 +703,7 @@
         <v>-0.02868596753592084</v>
       </c>
       <c r="C22" t="n">
-        <v>0.006499159944238406</v>
+        <v>-0.02868596753592084</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         <v>0.07310204929794104</v>
       </c>
       <c r="C23" t="n">
-        <v>0.02432290547365863</v>
+        <v>0.07310204929794104</v>
       </c>
     </row>
     <row r="24">
@@ -729,7 +729,7 @@
         <v>-0.008266017896256309</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.004043899313881078</v>
+        <v>-0.008266017896256309</v>
       </c>
     </row>
     <row r="25">
@@ -742,7 +742,7 @@
         <v>-0.02299908927089717</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.008342558226919244</v>
+        <v>-0.02299908927089717</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         <v>-0.04597418803989869</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.02629464696733087</v>
+        <v>-0.04597418803989869</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         <v>-0.0008416330670505273</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.00486581525864823</v>
+        <v>-0.0008416330670505273</v>
       </c>
     </row>
     <row r="28">
@@ -781,7 +781,7 @@
         <v>0.06982979119718163</v>
       </c>
       <c r="C28" t="n">
-        <v>0.06669128122946813</v>
+        <v>0.06982979119718163</v>
       </c>
     </row>
     <row r="29">
@@ -794,7 +794,7 @@
         <v>0.009758736779760392</v>
       </c>
       <c r="C29" t="n">
-        <v>-0.004283448597863186</v>
+        <v>0.009758736779760392</v>
       </c>
     </row>
     <row r="30">
@@ -807,7 +807,7 @@
         <v>0.007813680274738695</v>
       </c>
       <c r="C30" t="n">
-        <v>0.01352075931551485</v>
+        <v>0.007813680274738695</v>
       </c>
     </row>
     <row r="31">
@@ -820,7 +820,7 @@
         <v>-0.004728275154157093</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.007144770549359046</v>
+        <v>-0.004728275154157093</v>
       </c>
     </row>
     <row r="32">
@@ -833,7 +833,7 @@
         <v>0.03545544003008468</v>
       </c>
       <c r="C32" t="n">
-        <v>0.009598913515966879</v>
+        <v>0.03545544003008468</v>
       </c>
     </row>
     <row r="33">
@@ -846,7 +846,7 @@
         <v>-0.002665668212283876</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.003605949079416655</v>
+        <v>-0.002665668212283876</v>
       </c>
     </row>
     <row r="34">
@@ -859,7 +859,7 @@
         <v>0.004194882712985219</v>
       </c>
       <c r="C34" t="n">
-        <v>0.0001580415647026295</v>
+        <v>0.004194882712985219</v>
       </c>
     </row>
     <row r="35">
@@ -872,7 +872,7 @@
         <v>-0.02153205292396039</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.02910061731944192</v>
+        <v>-0.02153205292396039</v>
       </c>
     </row>
     <row r="36">
@@ -885,7 +885,7 @@
         <v>0.01404467658536659</v>
       </c>
       <c r="C36" t="n">
-        <v>0.01022999782199941</v>
+        <v>0.01404467658536659</v>
       </c>
     </row>
     <row r="37">
@@ -898,7 +898,7 @@
         <v>0.03183437725341597</v>
       </c>
       <c r="C37" t="n">
-        <v>0.02731912829651086</v>
+        <v>0.03183437725341597</v>
       </c>
     </row>
     <row r="38">
@@ -911,7 +911,7 @@
         <v>0.01740323486248268</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01506677803011915</v>
+        <v>0.01235380808043352</v>
       </c>
     </row>
     <row r="39">
@@ -924,7 +924,7 @@
         <v>0.02678288368048325</v>
       </c>
       <c r="C39" t="n">
-        <v>0.02657437106958093</v>
+        <v>0.0271228545104456</v>
       </c>
     </row>
     <row r="40">
@@ -937,7 +937,7 @@
         <v>0.01567374952350403</v>
       </c>
       <c r="C40" t="n">
-        <v>0.01719383153866666</v>
+        <v>0.01670126631426486</v>
       </c>
     </row>
     <row r="41">
@@ -950,7 +950,7 @@
         <v>0.01723994126614044</v>
       </c>
       <c r="C41" t="n">
-        <v>0.0283498480665103</v>
+        <v>0.02065721052381888</v>
       </c>
     </row>
     <row r="42">
@@ -963,7 +963,7 @@
         <v>0.02819533255836428</v>
       </c>
       <c r="C42" t="n">
-        <v>0.02592226137817534</v>
+        <v>0.02101957709536874</v>
       </c>
     </row>
     <row r="43">
@@ -976,7 +976,7 @@
         <v>-0.001645155946968475</v>
       </c>
       <c r="C43" t="n">
-        <v>0.01079968795946038</v>
+        <v>0.008520766898487358</v>
       </c>
     </row>
     <row r="44">
@@ -989,7 +989,7 @@
         <v>0.02242329502879963</v>
       </c>
       <c r="C44" t="n">
-        <v>0.01292604616584466</v>
+        <v>0.02156474586261202</v>
       </c>
     </row>
     <row r="45">
@@ -1002,7 +1002,7 @@
         <v>0.004444584316697018</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.01181849670132603</v>
+        <v>-0.006120973688339351</v>
       </c>
     </row>
     <row r="46">
@@ -1015,7 +1015,7 @@
         <v>0.02601056077789016</v>
       </c>
       <c r="C46" t="n">
-        <v>0.02641792497117698</v>
+        <v>0.01315578255227956</v>
       </c>
     </row>
     <row r="47">
@@ -1028,7 +1028,7 @@
         <v>0.01976264235981205</v>
       </c>
       <c r="C47" t="n">
-        <v>0.002196464589512326</v>
+        <v>0.006316413877071466</v>
       </c>
     </row>
     <row r="48">
@@ -1041,7 +1041,7 @@
         <v>0.02291278564579322</v>
       </c>
       <c r="C48" t="n">
-        <v>0.04254908936093235</v>
+        <v>0.0288431116194943</v>
       </c>
     </row>
     <row r="49">
@@ -1054,7 +1054,7 @@
         <v>0.01328848701450167</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01363015692617218</v>
+        <v>0.01153059554540475</v>
       </c>
     </row>
     <row r="50">
@@ -1067,7 +1067,7 @@
         <v>0.05450637476307812</v>
       </c>
       <c r="C50" t="n">
-        <v>0.03910636846886015</v>
+        <v>0.06786784209841226</v>
       </c>
     </row>
     <row r="51">
@@ -1080,7 +1080,7 @@
         <v>-0.04408659863341988</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.04559435790332688</v>
+        <v>-0.06250544292903337</v>
       </c>
     </row>
     <row r="52">
@@ -1093,7 +1093,7 @@
         <v>-0.01631617068573385</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.005913157870739245</v>
+        <v>-0.006972052722427907</v>
       </c>
     </row>
     <row r="53">
@@ -1106,7 +1106,7 @@
         <v>0.01311460741641066</v>
       </c>
       <c r="C53" t="n">
-        <v>0.002963630043256078</v>
+        <v>0.004066109447842278</v>
       </c>
     </row>
     <row r="54">
@@ -1119,7 +1119,7 @@
         <v>0.006591813712259888</v>
       </c>
       <c r="C54" t="n">
-        <v>0.01443896319432644</v>
+        <v>0.002875304851962855</v>
       </c>
     </row>
     <row r="55">
@@ -1132,7 +1132,7 @@
         <v>0.00282858753815986</v>
       </c>
       <c r="C55" t="n">
-        <v>0.0198933515196093</v>
+        <v>0.01481418793386685</v>
       </c>
     </row>
     <row r="56">
@@ -1145,7 +1145,7 @@
         <v>0.03841374457237075</v>
       </c>
       <c r="C56" t="n">
-        <v>0.02464784656280784</v>
+        <v>0.02495812530119474</v>
       </c>
     </row>
     <row r="57">
@@ -1158,7 +1158,7 @@
         <v>0.01613449834759624</v>
       </c>
       <c r="C57" t="n">
-        <v>0.02023630824362133</v>
+        <v>0.01084943975060963</v>
       </c>
     </row>
     <row r="58">
@@ -1171,7 +1171,7 @@
         <v>0.008135382599115809</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.007460860693777973</v>
+        <v>-0.003663787786282063</v>
       </c>
     </row>
     <row r="59">
@@ -1184,7 +1184,7 @@
         <v>-0.06824001451921091</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.04432000470100395</v>
+        <v>-0.04860347748449538</v>
       </c>
     </row>
     <row r="60">
@@ -1197,7 +1197,7 @@
         <v>0.009532010259542888</v>
       </c>
       <c r="C60" t="n">
-        <v>0.01644694235378497</v>
+        <v>0.02325474954312172</v>
       </c>
     </row>
     <row r="61">
@@ -1210,7 +1210,7 @@
         <v>-0.07513241411916755</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.05212498223691166</v>
+        <v>-0.05418482153182438</v>
       </c>
     </row>
     <row r="62">
@@ -1223,7 +1223,7 @@
         <v>0.07100953961674239</v>
       </c>
       <c r="C62" t="n">
-        <v>0.03203690307404896</v>
+        <v>0.07974815525811429</v>
       </c>
     </row>
     <row r="63">
@@ -1236,7 +1236,7 @@
         <v>0.03424002786314694</v>
       </c>
       <c r="C63" t="n">
-        <v>0.01941952458142587</v>
+        <v>0.03385936896805983</v>
       </c>
     </row>
     <row r="64">
@@ -1249,7 +1249,7 @@
         <v>0.01987483654089659</v>
       </c>
       <c r="C64" t="n">
-        <v>0.01165505023111339</v>
+        <v>0.02336167705323391</v>
       </c>
     </row>
     <row r="65">
@@ -1262,7 +1262,7 @@
         <v>0.03805610507780211</v>
       </c>
       <c r="C65" t="n">
-        <v>0.02471776209772535</v>
+        <v>0.03130650156387485</v>
       </c>
     </row>
     <row r="66">
@@ -1275,7 +1275,7 @@
         <v>-0.05763952152469834</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.01545098946956953</v>
+        <v>-0.0269331282453261</v>
       </c>
     </row>
     <row r="67">
@@ -1288,7 +1288,7 @@
         <v>0.07003192913895033</v>
       </c>
       <c r="C67" t="n">
-        <v>0.04305442878089966</v>
+        <v>0.05001760262875428</v>
       </c>
     </row>
     <row r="68">
@@ -1301,7 +1301,7 @@
         <v>0.005801666398690439</v>
       </c>
       <c r="C68" t="n">
-        <v>0.004273445160277805</v>
+        <v>0.01102441947674391</v>
       </c>
     </row>
     <row r="69">
@@ -1314,7 +1314,7 @@
         <v>-0.0119311832700844</v>
       </c>
       <c r="C69" t="n">
-        <v>0.005907611362144074</v>
+        <v>0.01129962966549056</v>
       </c>
     </row>
     <row r="70">
@@ -1327,7 +1327,7 @@
         <v>0.02046350005891205</v>
       </c>
       <c r="C70" t="n">
-        <v>0.008024839127055918</v>
+        <v>-0.001581481329794238</v>
       </c>
     </row>
     <row r="71">
@@ -1340,7 +1340,7 @@
         <v>0.01979282724021399</v>
       </c>
       <c r="C71" t="n">
-        <v>0.004234182076331864</v>
+        <v>0.01969619612332293</v>
       </c>
     </row>
     <row r="72">
@@ -1353,7 +1353,7 @@
         <v>0.02779959577757032</v>
       </c>
       <c r="C72" t="n">
-        <v>0.009960036500179554</v>
+        <v>0.01686586031941588</v>
       </c>
     </row>
     <row r="73">
@@ -1366,7 +1366,7 @@
         <v>0.03354079063457186</v>
       </c>
       <c r="C73" t="n">
-        <v>0.02268591000394431</v>
+        <v>0.04212203808782036</v>
       </c>
     </row>
     <row r="74">
@@ -1379,7 +1379,7 @@
         <v>-0.009512469421013588</v>
       </c>
       <c r="C74" t="n">
-        <v>0.005361029263695003</v>
+        <v>-0.01040580552949425</v>
       </c>
     </row>
     <row r="75">
@@ -1392,7 +1392,7 @@
         <v>-0.08873386778854889</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.08178524141402316</v>
+        <v>-0.09069053060445652</v>
       </c>
     </row>
     <row r="76">
@@ -1405,7 +1405,7 @@
         <v>-0.1316833338131493</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.09906993777483739</v>
+        <v>-0.1352120318892156</v>
       </c>
     </row>
     <row r="77">
@@ -1418,7 +1418,7 @@
         <v>0.1077626163796643</v>
       </c>
       <c r="C77" t="n">
-        <v>0.0008895280222904763</v>
+        <v>0.1220487561257171</v>
       </c>
     </row>
     <row r="78">
@@ -1431,7 +1431,7 @@
         <v>0.04054005034190309</v>
       </c>
       <c r="C78" t="n">
-        <v>0.03868235721395791</v>
+        <v>0.03682123859025232</v>
       </c>
     </row>
     <row r="79">
@@ -1444,7 +1444,7 @@
         <v>0.02696083125477164</v>
       </c>
       <c r="C79" t="n">
-        <v>0.001662100832240863</v>
+        <v>0.01297741872130764</v>
       </c>
     </row>
     <row r="80">
@@ -1457,7 +1457,7 @@
         <v>0.04943118353873739</v>
       </c>
       <c r="C80" t="n">
-        <v>0.01896547848066907</v>
+        <v>0.05865032517178752</v>
       </c>
     </row>
     <row r="81">
@@ -1470,7 +1470,7 @@
         <v>0.06408402856430478</v>
       </c>
       <c r="C81" t="n">
-        <v>0.03294979303070439</v>
+        <v>0.05820634999737539</v>
       </c>
     </row>
     <row r="82">
@@ -1483,7 +1483,7 @@
         <v>-0.03805992230318727</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.0145960946599522</v>
+        <v>-0.02678284458788993</v>
       </c>
     </row>
     <row r="83">
@@ -1496,7 +1496,7 @@
         <v>-0.03453704100332405</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.03164933509905492</v>
+        <v>-0.02498511709836092</v>
       </c>
     </row>
     <row r="84">
@@ -1509,7 +1509,7 @@
         <v>0.1284933508336998</v>
       </c>
       <c r="C84" t="n">
-        <v>0.03574114910400759</v>
+        <v>0.0997679999640611</v>
       </c>
     </row>
     <row r="85">
@@ -1522,7 +1522,7 @@
         <v>0.04144224819102368</v>
       </c>
       <c r="C85" t="n">
-        <v>0.03282520229528733</v>
+        <v>0.05100293901873042</v>
       </c>
     </row>
     <row r="86">
@@ -1535,7 +1535,7 @@
         <v>-0.01087269680571221</v>
       </c>
       <c r="C86" t="n">
-        <v>0.08877813413114544</v>
+        <v>-0.00270316554122419</v>
       </c>
     </row>
     <row r="87">
@@ -1548,7 +1548,7 @@
         <v>0.01726718854641026</v>
       </c>
       <c r="C87" t="n">
-        <v>-0.0335679862822223</v>
+        <v>0.00658166637473949</v>
       </c>
     </row>
     <row r="88">
@@ -1561,7 +1561,7 @@
         <v>0.04529814670424488</v>
       </c>
       <c r="C88" t="n">
-        <v>0.05047758021419248</v>
+        <v>0.05497080570908268</v>
       </c>
     </row>
     <row r="89">
@@ -1574,7 +1574,7 @@
         <v>0.0504471997770502</v>
       </c>
       <c r="C89" t="n">
-        <v>0.05183364502900376</v>
+        <v>0.03572355142819299</v>
       </c>
     </row>
     <row r="90">
@@ -1587,7 +1587,7 @@
         <v>0.01619715442258585</v>
       </c>
       <c r="C90" t="n">
-        <v>0.01862510225885376</v>
+        <v>0.02098657431143639</v>
       </c>
     </row>
     <row r="91">
@@ -1600,7 +1600,7 @@
         <v>0.0109283615463419</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.01268424424074623</v>
+        <v>0.0001113177313940518</v>
       </c>
     </row>
     <row r="92">
@@ -1613,7 +1613,7 @@
         <v>0.0245032958806435</v>
       </c>
       <c r="C92" t="n">
-        <v>0.04037330655556021</v>
+        <v>0.02512690604102937</v>
       </c>
     </row>
     <row r="93">
@@ -1626,7 +1626,7 @@
         <v>0.02218710615220952</v>
       </c>
       <c r="C93" t="n">
-        <v>0.008376307606520798</v>
+        <v>0.01039752070281994</v>
       </c>
     </row>
     <row r="94">
@@ -1639,7 +1639,7 @@
         <v>-0.05137128175717758</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.04773052087451022</v>
+        <v>-0.05406116741299745</v>
       </c>
     </row>
     <row r="95">
@@ -1652,7 +1652,7 @@
         <v>0.06403437245862154</v>
       </c>
       <c r="C95" t="n">
-        <v>0.03959031712719813</v>
+        <v>0.04496265449395401</v>
       </c>
     </row>
     <row r="96">
@@ -1665,7 +1665,7 @@
         <v>-0.0134136780319817</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.02782347383904496</v>
+        <v>-0.02110308289915133</v>
       </c>
     </row>
     <row r="97">
@@ -1678,7 +1678,7 @@
         <v>0.05573870955050739</v>
       </c>
       <c r="C97" t="n">
-        <v>0.06137376386370673</v>
+        <v>0.06276937323983428</v>
       </c>
     </row>
     <row r="98">
@@ -1691,7 +1691,7 @@
         <v>-0.04861561500165475</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.03445869753424048</v>
+        <v>-0.03888962702703988</v>
       </c>
     </row>
     <row r="99">
@@ -1704,7 +1704,7 @@
         <v>-0.02646097837535991</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.02282756066647776</v>
+        <v>-0.01729883536538741</v>
       </c>
     </row>
     <row r="100">
@@ -1717,7 +1717,7 @@
         <v>0.03272502952176156</v>
       </c>
       <c r="C100" t="n">
-        <v>0.05773639622080262</v>
+        <v>0.04470170774467979</v>
       </c>
     </row>
     <row r="101">
@@ -1730,7 +1730,7 @@
         <v>-0.07585617377799686</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.03381110686287254</v>
+        <v>-0.06180855856670836</v>
       </c>
     </row>
     <row r="102">
@@ -1743,7 +1743,7 @@
         <v>0.0009490514306432098</v>
       </c>
       <c r="C102" t="n">
-        <v>0.0133407653101496</v>
+        <v>0.006657086313991358</v>
       </c>
     </row>
     <row r="103">
@@ -1756,7 +1756,7 @@
         <v>-0.08170675120637592</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.04144327773357949</v>
+        <v>-0.06752159097856499</v>
       </c>
     </row>
     <row r="104">
@@ -1769,7 +1769,7 @@
         <v>0.08333980952073308</v>
       </c>
       <c r="C104" t="n">
-        <v>0.02656858605213656</v>
+        <v>0.06049294664513938</v>
       </c>
     </row>
     <row r="105">
@@ -1782,7 +1782,7 @@
         <v>-0.04578899609260523</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.02823600308526294</v>
+        <v>-0.03703070943076551</v>
       </c>
     </row>
     <row r="106">
@@ -1795,7 +1795,7 @@
         <v>-0.09191683746806092</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.0598897895645075</v>
+        <v>-0.08738035314436253</v>
       </c>
     </row>
     <row r="107">
@@ -1808,7 +1808,7 @@
         <v>0.07805033126155779</v>
       </c>
       <c r="C107" t="n">
-        <v>0.05162439959473308</v>
+        <v>0.07441252697703882</v>
       </c>
     </row>
     <row r="108">
@@ -1821,7 +1821,7 @@
         <v>0.06923963713672193</v>
       </c>
       <c r="C108" t="n">
-        <v>0.04507079789025119</v>
+        <v>0.06251444390463282</v>
       </c>
     </row>
     <row r="109">
@@ -1834,7 +1834,7 @@
         <v>-0.0437630907284597</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.03478965475231776</v>
+        <v>-0.03547778509646306</v>
       </c>
     </row>
     <row r="110">
@@ -1847,7 +1847,7 @@
         <v>0.06182610031980489</v>
       </c>
       <c r="C110" t="n">
-        <v>0.003903634849625049</v>
+        <v>0.04740931483648601</v>
       </c>
     </row>
     <row r="111">
@@ -1860,7 +1860,7 @@
         <v>-0.02363188778864639</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.03244715295620296</v>
+        <v>-0.02292438338867962</v>
       </c>
     </row>
     <row r="112">
@@ -1873,7 +1873,7 @@
         <v>0.03985696287954182</v>
       </c>
       <c r="C112" t="n">
-        <v>0.006929318166722013</v>
+        <v>0.02660600877376506</v>
       </c>
     </row>
     <row r="113">
@@ -1886,7 +1886,7 @@
         <v>0.02561957455128314</v>
       </c>
       <c r="C113" t="n">
-        <v>0.0393394143923302</v>
+        <v>0.02623403106987129</v>
       </c>
     </row>
     <row r="114">
@@ -1899,7 +1899,7 @@
         <v>-0.0144096424082673</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.04790684087229358</v>
+        <v>-0.02763350749328089</v>
       </c>
     </row>
     <row r="115">
@@ -1912,7 +1912,7 @@
         <v>0.06014567968316684</v>
       </c>
       <c r="C115" t="n">
-        <v>0.02082432852857487</v>
+        <v>0.03976441652019237</v>
       </c>
     </row>
     <row r="116">
@@ -1925,7 +1925,7 @@
         <v>0.02710549725651763</v>
       </c>
       <c r="C116" t="n">
-        <v>0.02401899367425473</v>
+        <v>0.02248472999244275</v>
       </c>
     </row>
     <row r="117">
@@ -1938,7 +1938,7 @@
         <v>-0.0219906500116242</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.03494236121370085</v>
+        <v>-0.01388397944447146</v>
       </c>
     </row>
     <row r="118">
@@ -1951,7 +1951,7 @@
         <v>-0.04806625468881839</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.02538415447936502</v>
+        <v>-0.04288821170594583</v>
       </c>
     </row>
     <row r="119">
@@ -1964,7 +1964,7 @@
         <v>-0.02479197802941527</v>
       </c>
       <c r="C119" t="n">
-        <v>0.0001082025444693176</v>
+        <v>-0.01902461699696891</v>
       </c>
     </row>
     <row r="120">
@@ -1977,7 +1977,7 @@
         <v>0.08931618762963371</v>
       </c>
       <c r="C120" t="n">
-        <v>0.04412675766711823</v>
+        <v>0.06205904269921394</v>
       </c>
     </row>
     <row r="121">
@@ -1990,7 +1990,7 @@
         <v>0.04431655704304508</v>
       </c>
       <c r="C121" t="n">
-        <v>-0.0009716219574559065</v>
+        <v>0.03231466666686127</v>
       </c>
     </row>
     <row r="122">
@@ -2003,7 +2003,7 @@
         <v>0.01313192008754371</v>
       </c>
       <c r="C122" t="n">
-        <v>0.01946129706733589</v>
+        <v>0.006904109312855763</v>
       </c>
     </row>
     <row r="123">
@@ -2016,7 +2016,7 @@
         <v>0.04147781442639268</v>
       </c>
       <c r="C123" t="n">
-        <v>0.03057874034580582</v>
+        <v>0.03364135334930279</v>
       </c>
     </row>
     <row r="124">
@@ -2029,7 +2029,7 @@
         <v>0.03176683813225063</v>
       </c>
       <c r="C124" t="n">
-        <v>0.01146870933054854</v>
+        <v>0.02773278653020967</v>
       </c>
     </row>
     <row r="125">
@@ -2042,7 +2042,7 @@
         <v>-0.03613653396606001</v>
       </c>
       <c r="C125" t="n">
-        <v>-0.0002756570360868994</v>
+        <v>-0.02019777135675051</v>
       </c>
     </row>
     <row r="126">
@@ -2055,7 +2055,7 @@
         <v>0.05356216202924662</v>
       </c>
       <c r="C126" t="n">
-        <v>0.03051250630379564</v>
+        <v>0.04127075433433336</v>
       </c>
     </row>
     <row r="127">
@@ -2068,7 +2068,7 @@
         <v>0.02064016352803047</v>
       </c>
       <c r="C127" t="n">
-        <v>0.00122399495049715</v>
+        <v>0.01295607953412005</v>
       </c>
     </row>
     <row r="128">
@@ -2081,7 +2081,7 @@
         <v>0.01341233672560688</v>
       </c>
       <c r="C128" t="n">
-        <v>0.04623631987883044</v>
+        <v>0.02170935259966802</v>
       </c>
     </row>
     <row r="129">
@@ -2094,7 +2094,7 @@
         <v>0.02677937050184446</v>
       </c>
       <c r="C129" t="n">
-        <v>0.03063001205915273</v>
+        <v>0.03580301115335468</v>
       </c>
     </row>
     <row r="130">
@@ -2107,7 +2107,7 @@
         <v>0.01453663215941871</v>
       </c>
       <c r="C130" t="n">
-        <v>-0.009963022349856285</v>
+        <v>0.003409084598160773</v>
       </c>
     </row>
     <row r="131">
@@ -2120,7 +2120,7 @@
         <v>-0.02352251844606836</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.007848104888712166</v>
+        <v>-0.04729543213552693</v>
       </c>
     </row>
     <row r="132">
@@ -2133,7 +2133,7 @@
         <v>0.04255994324570569</v>
       </c>
       <c r="C132" t="n">
-        <v>0.02368179766833487</v>
+        <v>0.0268816227250063</v>
       </c>
     </row>
     <row r="133">
@@ -2146,7 +2146,7 @@
         <v>-0.03202492799400349</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.0385509112011149</v>
+        <v>-0.03047851250570072</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add equal-weighted fallback portfolio and update SAAM presentation materials
</commit_message>
<xml_diff>
--- a/notebooks/monthly_portfolio_returns_2014_2025.xlsx
+++ b/notebooks/monthly_portfolio_returns_2014_2025.xlsx
@@ -911,7 +911,7 @@
         <v>0.01740323486248268</v>
       </c>
       <c r="C38" t="n">
-        <v>0.01235380808043352</v>
+        <v>0.02608683472897809</v>
       </c>
     </row>
     <row r="39">
@@ -924,7 +924,7 @@
         <v>0.02678288368048325</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0271228545104456</v>
+        <v>0.01540235791419027</v>
       </c>
     </row>
     <row r="40">
@@ -937,7 +937,7 @@
         <v>0.01567374952350403</v>
       </c>
       <c r="C40" t="n">
-        <v>0.01670126631426486</v>
+        <v>0.02158656537777273</v>
       </c>
     </row>
     <row r="41">
@@ -950,7 +950,7 @@
         <v>0.01723994126614044</v>
       </c>
       <c r="C41" t="n">
-        <v>0.02065721052381888</v>
+        <v>0.02712723590939563</v>
       </c>
     </row>
     <row r="42">
@@ -963,7 +963,7 @@
         <v>0.02819533255836428</v>
       </c>
       <c r="C42" t="n">
-        <v>0.02101957709536874</v>
+        <v>0.02205403990861593</v>
       </c>
     </row>
     <row r="43">
@@ -976,7 +976,7 @@
         <v>-0.001645155946968475</v>
       </c>
       <c r="C43" t="n">
-        <v>0.008520766898487358</v>
+        <v>0.003749176363448637</v>
       </c>
     </row>
     <row r="44">
@@ -989,7 +989,7 @@
         <v>0.02242329502879963</v>
       </c>
       <c r="C44" t="n">
-        <v>0.02156474586261202</v>
+        <v>0.02584462646495754</v>
       </c>
     </row>
     <row r="45">
@@ -1002,7 +1002,7 @@
         <v>0.004444584316697018</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.006120973688339351</v>
+        <v>-0.002882642896450579</v>
       </c>
     </row>
     <row r="46">
@@ -1015,7 +1015,7 @@
         <v>0.02601056077789016</v>
       </c>
       <c r="C46" t="n">
-        <v>0.01315578255227956</v>
+        <v>0.04122472453830364</v>
       </c>
     </row>
     <row r="47">
@@ -1028,7 +1028,7 @@
         <v>0.01976264235981205</v>
       </c>
       <c r="C47" t="n">
-        <v>0.006316413877071466</v>
+        <v>0.01087514076543347</v>
       </c>
     </row>
     <row r="48">
@@ -1041,7 +1041,7 @@
         <v>0.02291278564579322</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0288431116194943</v>
+        <v>0.02232321818738682</v>
       </c>
     </row>
     <row r="49">
@@ -1054,7 +1054,7 @@
         <v>0.01328848701450167</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01153059554540475</v>
+        <v>0.01782203367005048</v>
       </c>
     </row>
     <row r="50">
@@ -1067,7 +1067,7 @@
         <v>0.05450637476307812</v>
       </c>
       <c r="C50" t="n">
-        <v>0.06786784209841226</v>
+        <v>0.04751211742520459</v>
       </c>
     </row>
     <row r="51">
@@ -1080,7 +1080,7 @@
         <v>-0.04408659863341988</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.06250544292903337</v>
+        <v>-0.04960951442644493</v>
       </c>
     </row>
     <row r="52">
@@ -1093,7 +1093,7 @@
         <v>-0.01631617068573385</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.006972052722427907</v>
+        <v>-0.008434106680209007</v>
       </c>
     </row>
     <row r="53">
@@ -1106,7 +1106,7 @@
         <v>0.01311460741641066</v>
       </c>
       <c r="C53" t="n">
-        <v>0.004066109447842278</v>
+        <v>0.01929451225715609</v>
       </c>
     </row>
     <row r="54">
@@ -1119,7 +1119,7 @@
         <v>0.006591813712259888</v>
       </c>
       <c r="C54" t="n">
-        <v>0.002875304851962855</v>
+        <v>0.0007210133936334929</v>
       </c>
     </row>
     <row r="55">
@@ -1132,7 +1132,7 @@
         <v>0.00282858753815986</v>
       </c>
       <c r="C55" t="n">
-        <v>0.01481418793386685</v>
+        <v>-0.002698643204799356</v>
       </c>
     </row>
     <row r="56">
@@ -1145,7 +1145,7 @@
         <v>0.03841374457237075</v>
       </c>
       <c r="C56" t="n">
-        <v>0.02495812530119474</v>
+        <v>0.0268032863105044</v>
       </c>
     </row>
     <row r="57">
@@ -1158,7 +1158,7 @@
         <v>0.01613449834759624</v>
       </c>
       <c r="C57" t="n">
-        <v>0.01084943975060963</v>
+        <v>-0.0005943486201716031</v>
       </c>
     </row>
     <row r="58">
@@ -1171,7 +1171,7 @@
         <v>0.008135382599115809</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.003663787786282063</v>
+        <v>-0.002337924113460822</v>
       </c>
     </row>
     <row r="59">
@@ -1184,7 +1184,7 @@
         <v>-0.06824001451921091</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.04860347748449538</v>
+        <v>-0.0790812071277521</v>
       </c>
     </row>
     <row r="60">
@@ -1197,7 +1197,7 @@
         <v>0.009532010259542888</v>
       </c>
       <c r="C60" t="n">
-        <v>0.02325474954312172</v>
+        <v>0.006136017509973681</v>
       </c>
     </row>
     <row r="61">
@@ -1210,7 +1210,7 @@
         <v>-0.07513241411916755</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.05418482153182438</v>
+        <v>-0.07692745956218051</v>
       </c>
     </row>
     <row r="62">
@@ -1223,7 +1223,7 @@
         <v>0.07100953961674239</v>
       </c>
       <c r="C62" t="n">
-        <v>0.07974815525811429</v>
+        <v>0.09345517296877272</v>
       </c>
     </row>
     <row r="63">
@@ -1236,7 +1236,7 @@
         <v>0.03424002786314694</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03385936896805983</v>
+        <v>0.03540685742305543</v>
       </c>
     </row>
     <row r="64">
@@ -1249,7 +1249,7 @@
         <v>0.01987483654089659</v>
       </c>
       <c r="C64" t="n">
-        <v>0.02336167705323391</v>
+        <v>0.001332292368933422</v>
       </c>
     </row>
     <row r="65">
@@ -1262,7 +1262,7 @@
         <v>0.03805610507780211</v>
       </c>
       <c r="C65" t="n">
-        <v>0.03130650156387485</v>
+        <v>0.03918199654832371</v>
       </c>
     </row>
     <row r="66">
@@ -1275,7 +1275,7 @@
         <v>-0.05763952152469834</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.0269331282453261</v>
+        <v>-0.06692351481706189</v>
       </c>
     </row>
     <row r="67">
@@ -1288,7 +1288,7 @@
         <v>0.07003192913895033</v>
       </c>
       <c r="C67" t="n">
-        <v>0.05001760262875428</v>
+        <v>0.06441395216724799</v>
       </c>
     </row>
     <row r="68">
@@ -1301,7 +1301,7 @@
         <v>0.005801666398690439</v>
       </c>
       <c r="C68" t="n">
-        <v>0.01102441947674391</v>
+        <v>-0.008574934672832249</v>
       </c>
     </row>
     <row r="69">
@@ -1314,7 +1314,7 @@
         <v>-0.0119311832700844</v>
       </c>
       <c r="C69" t="n">
-        <v>0.01129962966549056</v>
+        <v>-0.03075880255029162</v>
       </c>
     </row>
     <row r="70">
@@ -1327,7 +1327,7 @@
         <v>0.02046350005891205</v>
       </c>
       <c r="C70" t="n">
-        <v>-0.001581481329794238</v>
+        <v>0.03326641514563633</v>
       </c>
     </row>
     <row r="71">
@@ -1340,7 +1340,7 @@
         <v>0.01979282724021399</v>
       </c>
       <c r="C71" t="n">
-        <v>0.01969619612332293</v>
+        <v>0.02330194870154663</v>
       </c>
     </row>
     <row r="72">
@@ -1353,7 +1353,7 @@
         <v>0.02779959577757032</v>
       </c>
       <c r="C72" t="n">
-        <v>0.01686586031941588</v>
+        <v>0.02921819917882855</v>
       </c>
     </row>
     <row r="73">
@@ -1366,7 +1366,7 @@
         <v>0.03354079063457186</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04212203808782036</v>
+        <v>0.04504811845933689</v>
       </c>
     </row>
     <row r="74">
@@ -1379,7 +1379,7 @@
         <v>-0.009512469421013588</v>
       </c>
       <c r="C74" t="n">
-        <v>-0.01040580552949425</v>
+        <v>-0.03086490561080929</v>
       </c>
     </row>
     <row r="75">
@@ -1392,7 +1392,7 @@
         <v>-0.08873386778854889</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.09069053060445652</v>
+        <v>-0.09718789127545738</v>
       </c>
     </row>
     <row r="76">
@@ -1405,7 +1405,7 @@
         <v>-0.1316833338131493</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.1352120318892156</v>
+        <v>-0.2205887820015016</v>
       </c>
     </row>
     <row r="77">
@@ -1418,7 +1418,7 @@
         <v>0.1077626163796643</v>
       </c>
       <c r="C77" t="n">
-        <v>0.1220487561257171</v>
+        <v>0.135770843339231</v>
       </c>
     </row>
     <row r="78">
@@ -1431,7 +1431,7 @@
         <v>0.04054005034190309</v>
       </c>
       <c r="C78" t="n">
-        <v>0.03682123859025232</v>
+        <v>0.04307186398182015</v>
       </c>
     </row>
     <row r="79">
@@ -1444,7 +1444,7 @@
         <v>0.02696083125477164</v>
       </c>
       <c r="C79" t="n">
-        <v>0.01297741872130764</v>
+        <v>0.02537534103768231</v>
       </c>
     </row>
     <row r="80">
@@ -1457,7 +1457,7 @@
         <v>0.04943118353873739</v>
       </c>
       <c r="C80" t="n">
-        <v>0.05865032517178752</v>
+        <v>0.04095652777442996</v>
       </c>
     </row>
     <row r="81">
@@ -1470,7 +1470,7 @@
         <v>0.06408402856430478</v>
       </c>
       <c r="C81" t="n">
-        <v>0.05820634999737539</v>
+        <v>0.05672231398115406</v>
       </c>
     </row>
     <row r="82">
@@ -1483,7 +1483,7 @@
         <v>-0.03805992230318727</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.02678284458788993</v>
+        <v>-0.04176369944637105</v>
       </c>
     </row>
     <row r="83">
@@ -1496,7 +1496,7 @@
         <v>-0.03453704100332405</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.02498511709836092</v>
+        <v>-0.01089159339051859</v>
       </c>
     </row>
     <row r="84">
@@ -1509,7 +1509,7 @@
         <v>0.1284933508336998</v>
       </c>
       <c r="C84" t="n">
-        <v>0.0997679999640611</v>
+        <v>0.2010399913398273</v>
       </c>
     </row>
     <row r="85">
@@ -1522,7 +1522,7 @@
         <v>0.04144224819102368</v>
       </c>
       <c r="C85" t="n">
-        <v>0.05100293901873042</v>
+        <v>0.05790893802921129</v>
       </c>
     </row>
     <row r="86">
@@ -1535,7 +1535,7 @@
         <v>-0.01087269680571221</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.00270316554122419</v>
+        <v>0.003149059754084705</v>
       </c>
     </row>
     <row r="87">
@@ -1548,7 +1548,7 @@
         <v>0.01726718854641026</v>
       </c>
       <c r="C87" t="n">
-        <v>0.00658166637473949</v>
+        <v>0.04435791506997791</v>
       </c>
     </row>
     <row r="88">
@@ -1561,7 +1561,7 @@
         <v>0.04529814670424488</v>
       </c>
       <c r="C88" t="n">
-        <v>0.05497080570908268</v>
+        <v>0.05039404201310474</v>
       </c>
     </row>
     <row r="89">
@@ -1574,7 +1574,7 @@
         <v>0.0504471997770502</v>
       </c>
       <c r="C89" t="n">
-        <v>0.03572355142819299</v>
+        <v>0.0475069377123306</v>
       </c>
     </row>
     <row r="90">
@@ -1587,7 +1587,7 @@
         <v>0.01619715442258585</v>
       </c>
       <c r="C90" t="n">
-        <v>0.02098657431143639</v>
+        <v>0.03629561654515578</v>
       </c>
     </row>
     <row r="91">
@@ -1600,7 +1600,7 @@
         <v>0.0109283615463419</v>
       </c>
       <c r="C91" t="n">
-        <v>0.0001113177313940518</v>
+        <v>-0.01652878039451288</v>
       </c>
     </row>
     <row r="92">
@@ -1613,7 +1613,7 @@
         <v>0.0245032958806435</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02512690604102937</v>
+        <v>0.02019047569277432</v>
       </c>
     </row>
     <row r="93">
@@ -1626,7 +1626,7 @@
         <v>0.02218710615220952</v>
       </c>
       <c r="C93" t="n">
-        <v>0.01039752070281994</v>
+        <v>0.01378237035208174</v>
       </c>
     </row>
     <row r="94">
@@ -1639,7 +1639,7 @@
         <v>-0.05137128175717758</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.05406116741299745</v>
+        <v>-0.0473121879703522</v>
       </c>
     </row>
     <row r="95">
@@ -1652,7 +1652,7 @@
         <v>0.06403437245862154</v>
       </c>
       <c r="C95" t="n">
-        <v>0.04496265449395401</v>
+        <v>0.04403864865034818</v>
       </c>
     </row>
     <row r="96">
@@ -1665,7 +1665,7 @@
         <v>-0.0134136780319817</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.02110308289915133</v>
+        <v>-0.03802285446390972</v>
       </c>
     </row>
     <row r="97">
@@ -1678,7 +1678,7 @@
         <v>0.05573870955050739</v>
       </c>
       <c r="C97" t="n">
-        <v>0.06276937323983428</v>
+        <v>0.06535599342100391</v>
       </c>
     </row>
     <row r="98">
@@ -1691,7 +1691,7 @@
         <v>-0.04861561500165475</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.03888962702703988</v>
+        <v>-0.04392791041261607</v>
       </c>
     </row>
     <row r="99">
@@ -1704,7 +1704,7 @@
         <v>-0.02646097837535991</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.01729883536538741</v>
+        <v>-0.01657793290611556</v>
       </c>
     </row>
     <row r="100">
@@ -1716,8 +1716,10 @@
       <c r="B100" t="n">
         <v>0.03272502952176156</v>
       </c>
-      <c r="C100" t="n">
-        <v>0.04470170774467979</v>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -1730,7 +1732,7 @@
         <v>-0.07585617377799686</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.06180855856670836</v>
+        <v>-0.05757797356300588</v>
       </c>
     </row>
     <row r="102">
@@ -1743,7 +1745,7 @@
         <v>0.0009490514306432098</v>
       </c>
       <c r="C102" t="n">
-        <v>0.006657086313991358</v>
+        <v>0.009864065878277047</v>
       </c>
     </row>
     <row r="103">
@@ -1756,7 +1758,7 @@
         <v>-0.08170675120637592</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.06752159097856499</v>
+        <v>-0.1006243422125562</v>
       </c>
     </row>
     <row r="104">
@@ -1769,7 +1771,7 @@
         <v>0.08333980952073308</v>
       </c>
       <c r="C104" t="n">
-        <v>0.06049294664513938</v>
+        <v>0.06907138122991631</v>
       </c>
     </row>
     <row r="105">
@@ -1782,7 +1784,7 @@
         <v>-0.04578899609260523</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.03703070943076551</v>
+        <v>-0.04935645726488558</v>
       </c>
     </row>
     <row r="106">
@@ -1795,7 +1797,7 @@
         <v>-0.09191683746806092</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.08738035314436253</v>
+        <v>-0.1001564999334072</v>
       </c>
     </row>
     <row r="107">
@@ -1808,7 +1810,7 @@
         <v>0.07805033126155779</v>
       </c>
       <c r="C107" t="n">
-        <v>0.07441252697703882</v>
+        <v>0.08829985514105151</v>
       </c>
     </row>
     <row r="108">
@@ -1821,7 +1823,7 @@
         <v>0.06923963713672193</v>
       </c>
       <c r="C108" t="n">
-        <v>0.06251444390463282</v>
+        <v>0.09256641307112776</v>
       </c>
     </row>
     <row r="109">
@@ -1834,7 +1836,7 @@
         <v>-0.0437630907284597</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.03547778509646306</v>
+        <v>-0.02120524177869844</v>
       </c>
     </row>
     <row r="110">
@@ -1847,7 +1849,7 @@
         <v>0.06182610031980489</v>
       </c>
       <c r="C110" t="n">
-        <v>0.04740931483648601</v>
+        <v>0.08649744905396635</v>
       </c>
     </row>
     <row r="111">
@@ -1860,7 +1862,7 @@
         <v>-0.02363188778864639</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.02292438338867962</v>
+        <v>-0.01720240828017944</v>
       </c>
     </row>
     <row r="112">
@@ -1873,7 +1875,7 @@
         <v>0.03985696287954182</v>
       </c>
       <c r="C112" t="n">
-        <v>0.02660600877376506</v>
+        <v>-0.005497931084551096</v>
       </c>
     </row>
     <row r="113">
@@ -1886,7 +1888,7 @@
         <v>0.02561957455128314</v>
       </c>
       <c r="C113" t="n">
-        <v>0.02623403106987129</v>
+        <v>0.01477196614366007</v>
       </c>
     </row>
     <row r="114">
@@ -1899,7 +1901,7 @@
         <v>-0.0144096424082673</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.02763350749328089</v>
+        <v>-0.04904696386521035</v>
       </c>
     </row>
     <row r="115">
@@ -1912,7 +1914,7 @@
         <v>0.06014567968316684</v>
       </c>
       <c r="C115" t="n">
-        <v>0.03976441652019237</v>
+        <v>0.05906467189514451</v>
       </c>
     </row>
     <row r="116">
@@ -1925,7 +1927,7 @@
         <v>0.02710549725651763</v>
       </c>
       <c r="C116" t="n">
-        <v>0.02248472999244275</v>
+        <v>0.04427829449168128</v>
       </c>
     </row>
     <row r="117">
@@ -1938,7 +1940,7 @@
         <v>-0.0219906500116242</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.01388397944447146</v>
+        <v>-0.03370108846692567</v>
       </c>
     </row>
     <row r="118">
@@ -1951,7 +1953,7 @@
         <v>-0.04806625468881839</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.04288821170594583</v>
+        <v>-0.04540832446980075</v>
       </c>
     </row>
     <row r="119">
@@ -1964,7 +1966,7 @@
         <v>-0.02479197802941527</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.01902461699696891</v>
+        <v>-0.04617084451111102</v>
       </c>
     </row>
     <row r="120">
@@ -1977,7 +1979,7 @@
         <v>0.08931618762963371</v>
       </c>
       <c r="C120" t="n">
-        <v>0.06205904269921394</v>
+        <v>0.09302830544563126</v>
       </c>
     </row>
     <row r="121">
@@ -1990,7 +1992,7 @@
         <v>0.04431655704304508</v>
       </c>
       <c r="C121" t="n">
-        <v>0.03231466666686127</v>
+        <v>0.06773938418548163</v>
       </c>
     </row>
     <row r="122">
@@ -2003,7 +2005,7 @@
         <v>0.01313192008754371</v>
       </c>
       <c r="C122" t="n">
-        <v>0.006904109312855763</v>
+        <v>-0.01803511544573584</v>
       </c>
     </row>
     <row r="123">
@@ -2015,8 +2017,10 @@
       <c r="B123" t="n">
         <v>0.04147781442639268</v>
       </c>
-      <c r="C123" t="n">
-        <v>0.03364135334930279</v>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -2029,7 +2033,7 @@
         <v>0.03176683813225063</v>
       </c>
       <c r="C124" t="n">
-        <v>0.02773278653020967</v>
+        <v>0.04143692255842578</v>
       </c>
     </row>
     <row r="125">
@@ -2042,7 +2046,7 @@
         <v>-0.03613653396606001</v>
       </c>
       <c r="C125" t="n">
-        <v>-0.02019777135675051</v>
+        <v>-0.02979810934100747</v>
       </c>
     </row>
     <row r="126">
@@ -2055,7 +2059,7 @@
         <v>0.05356216202924662</v>
       </c>
       <c r="C126" t="n">
-        <v>0.04127075433433336</v>
+        <v>0.04908135202587892</v>
       </c>
     </row>
     <row r="127">
@@ -2068,7 +2072,7 @@
         <v>0.02064016352803047</v>
       </c>
       <c r="C127" t="n">
-        <v>0.01295607953412005</v>
+        <v>-0.02942254204924746</v>
       </c>
     </row>
     <row r="128">
@@ -2081,7 +2085,7 @@
         <v>0.01341233672560688</v>
       </c>
       <c r="C128" t="n">
-        <v>0.02170935259966802</v>
+        <v>0.05506812810914476</v>
       </c>
     </row>
     <row r="129">
@@ -2094,7 +2098,7 @@
         <v>0.02677937050184446</v>
       </c>
       <c r="C129" t="n">
-        <v>0.03580301115335468</v>
+        <v>0.02122956255346637</v>
       </c>
     </row>
     <row r="130">
@@ -2107,7 +2111,7 @@
         <v>0.01453663215941871</v>
       </c>
       <c r="C130" t="n">
-        <v>0.003409084598160773</v>
+        <v>0.0194998238332747</v>
       </c>
     </row>
     <row r="131">
@@ -2120,7 +2124,7 @@
         <v>-0.02352251844606836</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.04729543213552693</v>
+        <v>-0.04311489559448421</v>
       </c>
     </row>
     <row r="132">
@@ -2133,7 +2137,7 @@
         <v>0.04255994324570569</v>
       </c>
       <c r="C132" t="n">
-        <v>0.0268816227250063</v>
+        <v>0.02568919439250861</v>
       </c>
     </row>
     <row r="133">
@@ -2146,7 +2150,7 @@
         <v>-0.03202492799400349</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.03047851250570072</v>
+        <v>-0.04702330726598303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update climate metrics and tracking error plots
</commit_message>
<xml_diff>
--- a/notebooks/monthly_portfolio_returns_2014_2025.xlsx
+++ b/notebooks/monthly_portfolio_returns_2014_2025.xlsx
@@ -1701,10 +1701,10 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>-0.02646097837535991</v>
+        <v>-0.02519509556925661</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.01657793290611556</v>
+        <v>-0.01651750301702887</v>
       </c>
     </row>
     <row r="100">
@@ -1714,12 +1714,10 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.03272502952176156</v>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>0.03319591481409771</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0.02123361333797682</v>
       </c>
     </row>
     <row r="101">
@@ -1729,10 +1727,10 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>-0.07585617377799686</v>
+        <v>-0.07576095823225454</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.05757797356300588</v>
+        <v>-0.05729812922005081</v>
       </c>
     </row>
     <row r="102">
@@ -1745,7 +1743,7 @@
         <v>0.0009490514306432098</v>
       </c>
       <c r="C102" t="n">
-        <v>0.009864065878277047</v>
+        <v>0.009816123881298787</v>
       </c>
     </row>
     <row r="103">
@@ -1758,7 +1756,7 @@
         <v>-0.08170675120637592</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.1006243422125562</v>
+        <v>-0.1001352810110371</v>
       </c>
     </row>
     <row r="104">
@@ -1771,7 +1769,7 @@
         <v>0.08333980952073308</v>
       </c>
       <c r="C104" t="n">
-        <v>0.06907138122991631</v>
+        <v>0.06873567585334321</v>
       </c>
     </row>
     <row r="105">
@@ -1781,10 +1779,10 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>-0.04578899609260523</v>
+        <v>-0.04574440971990758</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.04935645726488558</v>
+        <v>-0.04905660029486805</v>
       </c>
     </row>
     <row r="106">
@@ -1794,10 +1792,10 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>-0.09191683746806092</v>
+        <v>-0.09118543522674816</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.1001564999334072</v>
+        <v>-0.09930462204818984</v>
       </c>
     </row>
     <row r="107">
@@ -1807,10 +1805,10 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0.07805033126155779</v>
+        <v>0.07842283525794706</v>
       </c>
       <c r="C107" t="n">
-        <v>0.08829985514105151</v>
+        <v>0.08744153334138151</v>
       </c>
     </row>
     <row r="108">
@@ -1820,10 +1818,10 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>0.06923963713672193</v>
+        <v>0.06929546415745122</v>
       </c>
       <c r="C108" t="n">
-        <v>0.09256641307112776</v>
+        <v>0.09144166929140567</v>
       </c>
     </row>
     <row r="109">
@@ -1833,10 +1831,10 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>-0.0437630907284597</v>
+        <v>-0.04329073183121396</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02120524177869844</v>
+        <v>-0.02092181813402568</v>
       </c>
     </row>
     <row r="110">
@@ -1849,7 +1847,7 @@
         <v>0.06182610031980489</v>
       </c>
       <c r="C110" t="n">
-        <v>0.08649744905396635</v>
+        <v>0.08639687062483382</v>
       </c>
     </row>
     <row r="111">
@@ -1862,7 +1860,7 @@
         <v>-0.02363188778864639</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.01720240828017944</v>
+        <v>-0.01718240547985365</v>
       </c>
     </row>
     <row r="112">
@@ -1875,7 +1873,7 @@
         <v>0.03985696287954182</v>
       </c>
       <c r="C112" t="n">
-        <v>-0.005497931084551096</v>
+        <v>-0.005491538141429525</v>
       </c>
     </row>
     <row r="113">
@@ -1888,7 +1886,7 @@
         <v>0.02561957455128314</v>
       </c>
       <c r="C113" t="n">
-        <v>0.01477196614366007</v>
+        <v>0.01475478943884186</v>
       </c>
     </row>
     <row r="114">
@@ -1898,10 +1896,10 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>-0.0144096424082673</v>
+        <v>-0.01438141288809551</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.04904696386521035</v>
+        <v>-0.04893290115854707</v>
       </c>
     </row>
     <row r="115">
@@ -1911,10 +1909,10 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>0.06014567968316684</v>
+        <v>0.06023657756266654</v>
       </c>
       <c r="C115" t="n">
-        <v>0.05906467189514451</v>
+        <v>0.05885863234202192</v>
       </c>
     </row>
     <row r="116">
@@ -1927,7 +1925,7 @@
         <v>0.02710549725651763</v>
       </c>
       <c r="C116" t="n">
-        <v>0.04427829449168128</v>
+        <v>0.04412383532484983</v>
       </c>
     </row>
     <row r="117">
@@ -1940,7 +1938,7 @@
         <v>-0.0219906500116242</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.03370108846692567</v>
+        <v>-0.03358352653041313</v>
       </c>
     </row>
     <row r="118">
@@ -1953,7 +1951,7 @@
         <v>-0.04806625468881839</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.04540832446980075</v>
+        <v>-0.04524992333792935</v>
       </c>
     </row>
     <row r="119">
@@ -1963,10 +1961,10 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>-0.02479197802941527</v>
+        <v>-0.02255473753367339</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.04617084451111102</v>
+        <v>-0.04590240936860456</v>
       </c>
     </row>
     <row r="120">
@@ -1976,10 +1974,10 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>0.08931618762963371</v>
+        <v>0.08932403223703124</v>
       </c>
       <c r="C120" t="n">
-        <v>0.09302830544563126</v>
+        <v>0.0923792707564757</v>
       </c>
     </row>
     <row r="121">
@@ -1989,10 +1987,10 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>0.04431655704304508</v>
+        <v>0.04434459866854044</v>
       </c>
       <c r="C121" t="n">
-        <v>0.06773938418548163</v>
+        <v>0.06718801710490213</v>
       </c>
     </row>
     <row r="122">
@@ -2002,10 +2000,10 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>0.01313192008754371</v>
+        <v>0.0131319230141497</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.01803511544573584</v>
+        <v>-0.01801466746903999</v>
       </c>
     </row>
     <row r="123">
@@ -2017,10 +2015,8 @@
       <c r="B123" t="n">
         <v>0.04147781442639268</v>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="C123" t="n">
+        <v>0.01638332900704023</v>
       </c>
     </row>
     <row r="124">
@@ -2030,10 +2026,10 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>0.03176683813225063</v>
+        <v>0.03176687782497378</v>
       </c>
       <c r="C124" t="n">
-        <v>0.04143692255842578</v>
+        <v>0.04138994192060443</v>
       </c>
     </row>
     <row r="125">
@@ -2043,10 +2039,10 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>-0.03613653396606001</v>
+        <v>-0.03610871940813767</v>
       </c>
       <c r="C125" t="n">
-        <v>-0.02979810934100747</v>
+        <v>-0.02966297052313442</v>
       </c>
     </row>
     <row r="126">
@@ -2059,7 +2055,7 @@
         <v>0.05356216202924662</v>
       </c>
       <c r="C126" t="n">
-        <v>0.04908135202587892</v>
+        <v>0.04885876086022867</v>
       </c>
     </row>
     <row r="127">
@@ -2069,10 +2065,10 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>0.02064016352803047</v>
+        <v>0.02081663056902152</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.02942254204924746</v>
+        <v>-0.02922238870197367</v>
       </c>
     </row>
     <row r="128">
@@ -2082,10 +2078,10 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>0.01341233672560688</v>
+        <v>0.0137279502516987</v>
       </c>
       <c r="C128" t="n">
-        <v>0.05506812810914476</v>
+        <v>0.05450620843456166</v>
       </c>
     </row>
     <row r="129">
@@ -2098,7 +2094,7 @@
         <v>0.02677937050184446</v>
       </c>
       <c r="C129" t="n">
-        <v>0.02122956255346637</v>
+        <v>0.02101293436414529</v>
       </c>
     </row>
     <row r="130">
@@ -2108,10 +2104,10 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0.01453663215941871</v>
+        <v>0.0145366796150193</v>
       </c>
       <c r="C130" t="n">
-        <v>0.0194998238332747</v>
+        <v>0.01927873739525571</v>
       </c>
     </row>
     <row r="131">
@@ -2121,10 +2117,10 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>-0.02352251844606836</v>
+        <v>-0.02341961245173092</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.04311489559448421</v>
+        <v>-0.04257718147709268</v>
       </c>
     </row>
     <row r="132">
@@ -2134,10 +2130,10 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>0.04255994324570569</v>
+        <v>0.04268246661254674</v>
       </c>
       <c r="C132" t="n">
-        <v>0.02568919439250861</v>
+        <v>0.02533968154363095</v>
       </c>
     </row>
     <row r="133">
@@ -2150,7 +2146,7 @@
         <v>-0.03202492799400349</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.04702330726598303</v>
+        <v>-0.04638353437801047</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix carbon constrained portfolio and plotting
</commit_message>
<xml_diff>
--- a/notebooks/monthly_portfolio_returns_2014_2025.xlsx
+++ b/notebooks/monthly_portfolio_returns_2014_2025.xlsx
@@ -443,7 +443,7 @@
         <v>-0.03494855159817797</v>
       </c>
       <c r="C2" t="n">
-        <v>-0.03494855159817797</v>
+        <v>0.003929193363062062</v>
       </c>
     </row>
     <row r="3">
@@ -456,7 +456,7 @@
         <v>0.05470324098031322</v>
       </c>
       <c r="C3" t="n">
-        <v>0.05470324098031322</v>
+        <v>0.04816185991961708</v>
       </c>
     </row>
     <row r="4">
@@ -469,7 +469,7 @@
         <v>0.009290254635864935</v>
       </c>
       <c r="C4" t="n">
-        <v>0.009290254635864935</v>
+        <v>0.004175498868990745</v>
       </c>
     </row>
     <row r="5">
@@ -482,7 +482,7 @@
         <v>0.01705414331523906</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01705414331523906</v>
+        <v>0.009739531859848164</v>
       </c>
     </row>
     <row r="6">
@@ -495,7 +495,7 @@
         <v>0.01573781668140689</v>
       </c>
       <c r="C6" t="n">
-        <v>0.01573781668140689</v>
+        <v>0.0002594536806535863</v>
       </c>
     </row>
     <row r="7">
@@ -508,7 +508,7 @@
         <v>0.0135843254131045</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0135843254131045</v>
+        <v>0.01867762660797273</v>
       </c>
     </row>
     <row r="8">
@@ -521,7 +521,7 @@
         <v>-0.02297284055523763</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.02297284055523763</v>
+        <v>-0.02790178181521797</v>
       </c>
     </row>
     <row r="9">
@@ -534,7 +534,7 @@
         <v>0.02728537359108229</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02728537359108229</v>
+        <v>0.03888800417337648</v>
       </c>
     </row>
     <row r="10">
@@ -547,7 +547,7 @@
         <v>-0.02335601002647316</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.02335601002647316</v>
+        <v>-0.02735576667012935</v>
       </c>
     </row>
     <row r="11">
@@ -560,7 +560,7 @@
         <v>0.004632013532543199</v>
       </c>
       <c r="C11" t="n">
-        <v>0.004632013532543199</v>
+        <v>0.04190295655501688</v>
       </c>
     </row>
     <row r="12">
@@ -573,7 +573,7 @@
         <v>0.03041181054854081</v>
       </c>
       <c r="C12" t="n">
-        <v>0.03041181054854081</v>
+        <v>0.03069437477334842</v>
       </c>
     </row>
     <row r="13">
@@ -586,7 +586,7 @@
         <v>-0.01909033912522776</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.01909033912522776</v>
+        <v>0.01740951630734851</v>
       </c>
     </row>
     <row r="14">
@@ -599,7 +599,7 @@
         <v>-0.01938885162887482</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.01938885162887482</v>
+        <v>-0.0116336921843984</v>
       </c>
     </row>
     <row r="15">
@@ -612,7 +612,7 @@
         <v>0.05742801269246856</v>
       </c>
       <c r="C15" t="n">
-        <v>0.05742801269246856</v>
+        <v>0.02735037725364751</v>
       </c>
     </row>
     <row r="16">
@@ -625,7 +625,7 @@
         <v>-0.01823988426294667</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.01823988426294667</v>
+        <v>-0.009505115112305571</v>
       </c>
     </row>
     <row r="17">
@@ -638,7 +638,7 @@
         <v>0.02302326507590106</v>
       </c>
       <c r="C17" t="n">
-        <v>0.02302326507590106</v>
+        <v>0.006294930583162122</v>
       </c>
     </row>
     <row r="18">
@@ -651,7 +651,7 @@
         <v>0.001559662658366811</v>
       </c>
       <c r="C18" t="n">
-        <v>0.001559662658366811</v>
+        <v>-0.005372193226347251</v>
       </c>
     </row>
     <row r="19">
@@ -664,7 +664,7 @@
         <v>-0.02756496175961278</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.02756496175961278</v>
+        <v>-0.02870440520319284</v>
       </c>
     </row>
     <row r="20">
@@ -677,7 +677,7 @@
         <v>0.02337215247765667</v>
       </c>
       <c r="C20" t="n">
-        <v>0.02337215247765667</v>
+        <v>0.0464589065352374</v>
       </c>
     </row>
     <row r="21">
@@ -690,7 +690,7 @@
         <v>-0.0622245390646549</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.0622245390646549</v>
+        <v>-0.04566495879118411</v>
       </c>
     </row>
     <row r="22">
@@ -703,7 +703,7 @@
         <v>-0.02868596753592084</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.02868596753592084</v>
+        <v>-0.02352145523807737</v>
       </c>
     </row>
     <row r="23">
@@ -716,7 +716,7 @@
         <v>0.07310204929794104</v>
       </c>
       <c r="C23" t="n">
-        <v>0.07310204929794104</v>
+        <v>0.02321061519355638</v>
       </c>
     </row>
     <row r="24">
@@ -729,7 +729,7 @@
         <v>-0.008266017896256309</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.008266017896256309</v>
+        <v>0.001234255141605822</v>
       </c>
     </row>
     <row r="25">
@@ -742,7 +742,7 @@
         <v>-0.02299908927089717</v>
       </c>
       <c r="C25" t="n">
-        <v>-0.02299908927089717</v>
+        <v>0.000102545121362734</v>
       </c>
     </row>
     <row r="26">
@@ -755,7 +755,7 @@
         <v>-0.04597418803989869</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.04597418803989869</v>
+        <v>-0.007259951525716971</v>
       </c>
     </row>
     <row r="27">
@@ -768,7 +768,7 @@
         <v>-0.0008416330670505273</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.0008416330670505273</v>
+        <v>-0.008219906607929785</v>
       </c>
     </row>
     <row r="28">
@@ -781,7 +781,7 @@
         <v>0.06982979119718163</v>
       </c>
       <c r="C28" t="n">
-        <v>0.06982979119718163</v>
+        <v>0.05741118057516965</v>
       </c>
     </row>
     <row r="29">
@@ -794,7 +794,7 @@
         <v>0.009758736779760392</v>
       </c>
       <c r="C29" t="n">
-        <v>0.009758736779760392</v>
+        <v>0.01074687273990775</v>
       </c>
     </row>
     <row r="30">
@@ -807,7 +807,7 @@
         <v>0.007813680274738695</v>
       </c>
       <c r="C30" t="n">
-        <v>0.007813680274738695</v>
+        <v>0.003999804756221921</v>
       </c>
     </row>
     <row r="31">
@@ -820,7 +820,7 @@
         <v>-0.004728275154157093</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.004728275154157093</v>
+        <v>0.03710683112036362</v>
       </c>
     </row>
     <row r="32">
@@ -833,7 +833,7 @@
         <v>0.03545544003008468</v>
       </c>
       <c r="C32" t="n">
-        <v>0.03545544003008468</v>
+        <v>0.02035906842021824</v>
       </c>
     </row>
     <row r="33">
@@ -846,7 +846,7 @@
         <v>-0.002665668212283876</v>
       </c>
       <c r="C33" t="n">
-        <v>-0.002665668212283876</v>
+        <v>-0.05725351925224963</v>
       </c>
     </row>
     <row r="34">
@@ -859,7 +859,7 @@
         <v>0.004194882712985219</v>
       </c>
       <c r="C34" t="n">
-        <v>0.004194882712985219</v>
+        <v>-0.006060409492049978</v>
       </c>
     </row>
     <row r="35">
@@ -872,7 +872,7 @@
         <v>-0.02153205292396039</v>
       </c>
       <c r="C35" t="n">
-        <v>-0.02153205292396039</v>
+        <v>-0.005654410612478939</v>
       </c>
     </row>
     <row r="36">
@@ -885,7 +885,7 @@
         <v>0.01404467658536659</v>
       </c>
       <c r="C36" t="n">
-        <v>0.01404467658536659</v>
+        <v>0.009210156471418318</v>
       </c>
     </row>
     <row r="37">
@@ -898,7 +898,7 @@
         <v>0.03183437725341597</v>
       </c>
       <c r="C37" t="n">
-        <v>0.03183437725341597</v>
+        <v>0.009734819944780041</v>
       </c>
     </row>
     <row r="38">
@@ -911,7 +911,7 @@
         <v>0.01740323486248268</v>
       </c>
       <c r="C38" t="n">
-        <v>0.02608683472897809</v>
+        <v>0.007304381298384354</v>
       </c>
     </row>
     <row r="39">
@@ -924,7 +924,7 @@
         <v>0.02678288368048325</v>
       </c>
       <c r="C39" t="n">
-        <v>0.01540235791419027</v>
+        <v>0.02746282534040796</v>
       </c>
     </row>
     <row r="40">
@@ -937,7 +937,7 @@
         <v>0.01567374952350403</v>
       </c>
       <c r="C40" t="n">
-        <v>0.02158656537777273</v>
+        <v>0.01772878310502569</v>
       </c>
     </row>
     <row r="41">
@@ -950,7 +950,7 @@
         <v>0.01723994126614044</v>
       </c>
       <c r="C41" t="n">
-        <v>0.02712723590939563</v>
+        <v>0.02407447978149731</v>
       </c>
     </row>
     <row r="42">
@@ -963,7 +963,7 @@
         <v>0.02819533255836428</v>
       </c>
       <c r="C42" t="n">
-        <v>0.02205403990861593</v>
+        <v>0.0138438216323732</v>
       </c>
     </row>
     <row r="43">
@@ -976,7 +976,7 @@
         <v>-0.001645155946968475</v>
       </c>
       <c r="C43" t="n">
-        <v>0.003749176363448637</v>
+        <v>0.01868668974394319</v>
       </c>
     </row>
     <row r="44">
@@ -989,7 +989,7 @@
         <v>0.02242329502879963</v>
       </c>
       <c r="C44" t="n">
-        <v>0.02584462646495754</v>
+        <v>0.02070619669642442</v>
       </c>
     </row>
     <row r="45">
@@ -1002,7 +1002,7 @@
         <v>0.004444584316697018</v>
       </c>
       <c r="C45" t="n">
-        <v>-0.002882642896450579</v>
+        <v>-0.01668653169337572</v>
       </c>
     </row>
     <row r="46">
@@ -1015,7 +1015,7 @@
         <v>0.02601056077789016</v>
       </c>
       <c r="C46" t="n">
-        <v>0.04122472453830364</v>
+        <v>0.0003010043266689549</v>
       </c>
     </row>
     <row r="47">
@@ -1028,7 +1028,7 @@
         <v>0.01976264235981205</v>
       </c>
       <c r="C47" t="n">
-        <v>0.01087514076543347</v>
+        <v>-0.007129814605669114</v>
       </c>
     </row>
     <row r="48">
@@ -1041,7 +1041,7 @@
         <v>0.02291278564579322</v>
       </c>
       <c r="C48" t="n">
-        <v>0.02232321818738682</v>
+        <v>0.03477343759319538</v>
       </c>
     </row>
     <row r="49">
@@ -1054,7 +1054,7 @@
         <v>0.01328848701450167</v>
       </c>
       <c r="C49" t="n">
-        <v>0.01782203367005048</v>
+        <v>0.009772704076307839</v>
       </c>
     </row>
     <row r="50">
@@ -1067,7 +1067,7 @@
         <v>0.05450637476307812</v>
       </c>
       <c r="C50" t="n">
-        <v>0.04751211742520459</v>
+        <v>0.0812293094337464</v>
       </c>
     </row>
     <row r="51">
@@ -1080,7 +1080,7 @@
         <v>-0.04408659863341988</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.04960951442644493</v>
+        <v>-0.08092428722464685</v>
       </c>
     </row>
     <row r="52">
@@ -1093,7 +1093,7 @@
         <v>-0.01631617068573385</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.008434106680209007</v>
+        <v>0.002372065240878036</v>
       </c>
     </row>
     <row r="53">
@@ -1106,7 +1106,7 @@
         <v>0.01311460741641066</v>
       </c>
       <c r="C53" t="n">
-        <v>0.01929451225715609</v>
+        <v>-0.004982388520726107</v>
       </c>
     </row>
     <row r="54">
@@ -1119,7 +1119,7 @@
         <v>0.006591813712259888</v>
       </c>
       <c r="C54" t="n">
-        <v>0.0007210133936334929</v>
+        <v>-0.0008412040083341781</v>
       </c>
     </row>
     <row r="55">
@@ -1132,7 +1132,7 @@
         <v>0.00282858753815986</v>
       </c>
       <c r="C55" t="n">
-        <v>-0.002698643204799356</v>
+        <v>0.02679978832957384</v>
       </c>
     </row>
     <row r="56">
@@ -1145,7 +1145,7 @@
         <v>0.03841374457237075</v>
       </c>
       <c r="C56" t="n">
-        <v>0.0268032863105044</v>
+        <v>0.01150250603001874</v>
       </c>
     </row>
     <row r="57">
@@ -1158,7 +1158,7 @@
         <v>0.01613449834759624</v>
       </c>
       <c r="C57" t="n">
-        <v>-0.0005943486201716031</v>
+        <v>0.005564381153623027</v>
       </c>
     </row>
     <row r="58">
@@ -1171,7 +1171,7 @@
         <v>0.008135382599115809</v>
       </c>
       <c r="C58" t="n">
-        <v>-0.002337924113460822</v>
+        <v>-0.01546295817167993</v>
       </c>
     </row>
     <row r="59">
@@ -1184,7 +1184,7 @@
         <v>-0.06824001451921091</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.0790812071277521</v>
+        <v>-0.02896694044977985</v>
       </c>
     </row>
     <row r="60">
@@ -1197,7 +1197,7 @@
         <v>0.009532010259542888</v>
       </c>
       <c r="C60" t="n">
-        <v>0.006136017509973681</v>
+        <v>0.03697748882670055</v>
       </c>
     </row>
     <row r="61">
@@ -1210,7 +1210,7 @@
         <v>-0.07513241411916755</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.07692745956218051</v>
+        <v>-0.03323722894448123</v>
       </c>
     </row>
     <row r="62">
@@ -1223,7 +1223,7 @@
         <v>0.07100953961674239</v>
       </c>
       <c r="C62" t="n">
-        <v>0.09345517296877272</v>
+        <v>0.0884867708994862</v>
       </c>
     </row>
     <row r="63">
@@ -1236,7 +1236,7 @@
         <v>0.03424002786314694</v>
       </c>
       <c r="C63" t="n">
-        <v>0.03540685742305543</v>
+        <v>0.03347871007297272</v>
       </c>
     </row>
     <row r="64">
@@ -1249,7 +1249,7 @@
         <v>0.01987483654089659</v>
       </c>
       <c r="C64" t="n">
-        <v>0.001332292368933422</v>
+        <v>0.02684851756557122</v>
       </c>
     </row>
     <row r="65">
@@ -1262,7 +1262,7 @@
         <v>0.03805610507780211</v>
       </c>
       <c r="C65" t="n">
-        <v>0.03918199654832371</v>
+        <v>0.02455689804994758</v>
       </c>
     </row>
     <row r="66">
@@ -1275,7 +1275,7 @@
         <v>-0.05763952152469834</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.06692351481706189</v>
+        <v>0.003773265034046149</v>
       </c>
     </row>
     <row r="67">
@@ -1288,7 +1288,7 @@
         <v>0.07003192913895033</v>
       </c>
       <c r="C67" t="n">
-        <v>0.06441395216724799</v>
+        <v>0.03000327611855823</v>
       </c>
     </row>
     <row r="68">
@@ -1301,7 +1301,7 @@
         <v>0.005801666398690439</v>
       </c>
       <c r="C68" t="n">
-        <v>-0.008574934672832249</v>
+        <v>0.01624717255479739</v>
       </c>
     </row>
     <row r="69">
@@ -1314,7 +1314,7 @@
         <v>-0.0119311832700844</v>
       </c>
       <c r="C69" t="n">
-        <v>-0.03075880255029162</v>
+        <v>0.03453044260106552</v>
       </c>
     </row>
     <row r="70">
@@ -1327,7 +1327,7 @@
         <v>0.02046350005891205</v>
       </c>
       <c r="C70" t="n">
-        <v>0.03326641514563633</v>
+        <v>-0.02362646271850053</v>
       </c>
     </row>
     <row r="71">
@@ -1340,7 +1340,7 @@
         <v>0.01979282724021399</v>
       </c>
       <c r="C71" t="n">
-        <v>0.02330194870154663</v>
+        <v>0.01959956500643188</v>
       </c>
     </row>
     <row r="72">
@@ -1353,7 +1353,7 @@
         <v>0.02779959577757032</v>
       </c>
       <c r="C72" t="n">
-        <v>0.02921819917882855</v>
+        <v>0.005932124861261435</v>
       </c>
     </row>
     <row r="73">
@@ -1366,7 +1366,7 @@
         <v>0.03354079063457186</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04504811845933689</v>
+        <v>0.05070328554106886</v>
       </c>
     </row>
     <row r="74">
@@ -1379,7 +1379,7 @@
         <v>-0.009512469421013588</v>
       </c>
       <c r="C74" t="n">
-        <v>-0.03086490561080929</v>
+        <v>-0.01129914163797492</v>
       </c>
     </row>
     <row r="75">
@@ -1392,7 +1392,7 @@
         <v>-0.08873386778854889</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.09718789127545738</v>
+        <v>-0.09264719342036415</v>
       </c>
     </row>
     <row r="76">
@@ -1405,7 +1405,7 @@
         <v>-0.1316833338131493</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.2205887820015016</v>
+        <v>-0.1387407299652818</v>
       </c>
     </row>
     <row r="77">
@@ -1418,7 +1418,7 @@
         <v>0.1077626163796643</v>
       </c>
       <c r="C77" t="n">
-        <v>0.135770843339231</v>
+        <v>0.13633489587177</v>
       </c>
     </row>
     <row r="78">
@@ -1431,7 +1431,7 @@
         <v>0.04054005034190309</v>
       </c>
       <c r="C78" t="n">
-        <v>0.04307186398182015</v>
+        <v>0.03310242683860155</v>
       </c>
     </row>
     <row r="79">
@@ -1444,7 +1444,7 @@
         <v>0.02696083125477164</v>
       </c>
       <c r="C79" t="n">
-        <v>0.02537534103768231</v>
+        <v>-0.001005993812156355</v>
       </c>
     </row>
     <row r="80">
@@ -1457,7 +1457,7 @@
         <v>0.04943118353873739</v>
       </c>
       <c r="C80" t="n">
-        <v>0.04095652777442996</v>
+        <v>0.06786946680483764</v>
       </c>
     </row>
     <row r="81">
@@ -1470,7 +1470,7 @@
         <v>0.06408402856430478</v>
       </c>
       <c r="C81" t="n">
-        <v>0.05672231398115406</v>
+        <v>0.05232867143044599</v>
       </c>
     </row>
     <row r="82">
@@ -1483,7 +1483,7 @@
         <v>-0.03805992230318727</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.04176369944637105</v>
+        <v>-0.01550576687259259</v>
       </c>
     </row>
     <row r="83">
@@ -1496,7 +1496,7 @@
         <v>-0.03453704100332405</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.01089159339051859</v>
+        <v>-0.01543319319339779</v>
       </c>
     </row>
     <row r="84">
@@ -1509,7 +1509,7 @@
         <v>0.1284933508336998</v>
       </c>
       <c r="C84" t="n">
-        <v>0.2010399913398273</v>
+        <v>0.07104264909442241</v>
       </c>
     </row>
     <row r="85">
@@ -1522,7 +1522,7 @@
         <v>0.04144224819102368</v>
       </c>
       <c r="C85" t="n">
-        <v>0.05790893802921129</v>
+        <v>0.06056362984643716</v>
       </c>
     </row>
     <row r="86">
@@ -1535,7 +1535,7 @@
         <v>-0.01087269680571221</v>
       </c>
       <c r="C86" t="n">
-        <v>0.003149059754084705</v>
+        <v>0.005466365723263833</v>
       </c>
     </row>
     <row r="87">
@@ -1548,7 +1548,7 @@
         <v>0.01726718854641026</v>
       </c>
       <c r="C87" t="n">
-        <v>0.04435791506997791</v>
+        <v>-0.004103855796931283</v>
       </c>
     </row>
     <row r="88">
@@ -1561,7 +1561,7 @@
         <v>0.04529814670424488</v>
       </c>
       <c r="C88" t="n">
-        <v>0.05039404201310474</v>
+        <v>0.06464346471392048</v>
       </c>
     </row>
     <row r="89">
@@ -1574,7 +1574,7 @@
         <v>0.0504471997770502</v>
       </c>
       <c r="C89" t="n">
-        <v>0.0475069377123306</v>
+        <v>0.02099990307933578</v>
       </c>
     </row>
     <row r="90">
@@ -1587,7 +1587,7 @@
         <v>0.01619715442258585</v>
       </c>
       <c r="C90" t="n">
-        <v>0.03629561654515578</v>
+        <v>0.02577599420028694</v>
       </c>
     </row>
     <row r="91">
@@ -1600,7 +1600,7 @@
         <v>0.0109283615463419</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.01652878039451288</v>
+        <v>-0.01070572608355379</v>
       </c>
     </row>
     <row r="92">
@@ -1613,7 +1613,7 @@
         <v>0.0245032958806435</v>
       </c>
       <c r="C92" t="n">
-        <v>0.02019047569277432</v>
+        <v>0.02575051620141524</v>
       </c>
     </row>
     <row r="93">
@@ -1626,7 +1626,7 @@
         <v>0.02218710615220952</v>
       </c>
       <c r="C93" t="n">
-        <v>0.01378237035208174</v>
+        <v>-0.001392064746569636</v>
       </c>
     </row>
     <row r="94">
@@ -1639,7 +1639,7 @@
         <v>-0.05137128175717758</v>
       </c>
       <c r="C94" t="n">
-        <v>-0.0473121879703522</v>
+        <v>-0.05675105306881732</v>
       </c>
     </row>
     <row r="95">
@@ -1652,7 +1652,7 @@
         <v>0.06403437245862154</v>
       </c>
       <c r="C95" t="n">
-        <v>0.04403864865034818</v>
+        <v>0.02589093652928648</v>
       </c>
     </row>
     <row r="96">
@@ -1665,7 +1665,7 @@
         <v>-0.0134136780319817</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.03802285446390972</v>
+        <v>-0.02879248776632095</v>
       </c>
     </row>
     <row r="97">
@@ -1678,7 +1678,7 @@
         <v>0.05573870955050739</v>
       </c>
       <c r="C97" t="n">
-        <v>0.06535599342100391</v>
+        <v>0.06980003692916119</v>
       </c>
     </row>
     <row r="98">
@@ -1691,7 +1691,7 @@
         <v>-0.04861561500165475</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.04392791041261607</v>
+        <v>-0.02916363905242501</v>
       </c>
     </row>
     <row r="99">
@@ -1704,7 +1704,7 @@
         <v>-0.02519509556925661</v>
       </c>
       <c r="C99" t="n">
-        <v>-0.01651750301702887</v>
+        <v>-0.008136692355414914</v>
       </c>
     </row>
     <row r="100">
@@ -1717,7 +1717,7 @@
         <v>0.03319591481409771</v>
       </c>
       <c r="C100" t="n">
-        <v>0.02123361333797682</v>
+        <v>0.05667838596759802</v>
       </c>
     </row>
     <row r="101">
@@ -1730,7 +1730,7 @@
         <v>-0.07576095823225454</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.05729812922005081</v>
+        <v>-0.04776094335541986</v>
       </c>
     </row>
     <row r="102">
@@ -1743,7 +1743,7 @@
         <v>0.0009490514306432098</v>
       </c>
       <c r="C102" t="n">
-        <v>0.009816123881298787</v>
+        <v>0.01236512119733951</v>
       </c>
     </row>
     <row r="103">
@@ -1756,7 +1756,7 @@
         <v>-0.08170675120637592</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.1001352810110371</v>
+        <v>-0.05333643075075405</v>
       </c>
     </row>
     <row r="104">
@@ -1769,7 +1769,7 @@
         <v>0.08333980952073308</v>
       </c>
       <c r="C104" t="n">
-        <v>0.06873567585334321</v>
+        <v>0.03764608376954568</v>
       </c>
     </row>
     <row r="105">
@@ -1782,7 +1782,7 @@
         <v>-0.04574440971990758</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.04905660029486805</v>
+        <v>-0.02827242276892579</v>
       </c>
     </row>
     <row r="106">
@@ -1795,7 +1795,7 @@
         <v>-0.09118543522674816</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.09930462204818984</v>
+        <v>-0.08284386882066413</v>
       </c>
     </row>
     <row r="107">
@@ -1808,7 +1808,7 @@
         <v>0.07842283525794706</v>
       </c>
       <c r="C107" t="n">
-        <v>0.08744153334138151</v>
+        <v>0.07077472269251983</v>
       </c>
     </row>
     <row r="108">
@@ -1821,7 +1821,7 @@
         <v>0.06929546415745122</v>
       </c>
       <c r="C108" t="n">
-        <v>0.09144166929140567</v>
+        <v>0.05578925067254371</v>
       </c>
     </row>
     <row r="109">
@@ -1834,7 +1834,7 @@
         <v>-0.04329073183121396</v>
       </c>
       <c r="C109" t="n">
-        <v>-0.02092181813402568</v>
+        <v>-0.02719247946446643</v>
       </c>
     </row>
     <row r="110">
@@ -1847,7 +1847,7 @@
         <v>0.06182610031980489</v>
       </c>
       <c r="C110" t="n">
-        <v>0.08639687062483382</v>
+        <v>0.03299252935316713</v>
       </c>
     </row>
     <row r="111">
@@ -1860,7 +1860,7 @@
         <v>-0.02363188778864639</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.01718240547985365</v>
+        <v>-0.02221687898871285</v>
       </c>
     </row>
     <row r="112">
@@ -1873,7 +1873,7 @@
         <v>0.03985696287954182</v>
       </c>
       <c r="C112" t="n">
-        <v>-0.005491538141429525</v>
+        <v>0.0133550546679883</v>
       </c>
     </row>
     <row r="113">
@@ -1886,7 +1886,7 @@
         <v>0.02561957455128314</v>
       </c>
       <c r="C113" t="n">
-        <v>0.01475478943884186</v>
+        <v>0.02684848758845945</v>
       </c>
     </row>
     <row r="114">
@@ -1899,7 +1899,7 @@
         <v>-0.01438141288809551</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.04893290115854707</v>
+        <v>-0.04085737257829449</v>
       </c>
     </row>
     <row r="115">
@@ -1912,7 +1912,7 @@
         <v>0.06023657756266654</v>
       </c>
       <c r="C115" t="n">
-        <v>0.05885863234202192</v>
+        <v>0.01938315335721791</v>
       </c>
     </row>
     <row r="116">
@@ -1925,7 +1925,7 @@
         <v>0.02710549725651763</v>
       </c>
       <c r="C116" t="n">
-        <v>0.04412383532484983</v>
+        <v>0.01786396272836788</v>
       </c>
     </row>
     <row r="117">
@@ -1938,7 +1938,7 @@
         <v>-0.0219906500116242</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.03358352653041313</v>
+        <v>-0.005777308877318728</v>
       </c>
     </row>
     <row r="118">
@@ -1951,7 +1951,7 @@
         <v>-0.04806625468881839</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.04524992333792935</v>
+        <v>-0.03771016872307327</v>
       </c>
     </row>
     <row r="119">
@@ -1964,7 +1964,7 @@
         <v>-0.02255473753367339</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.04590240936860456</v>
+        <v>-0.01325725596452254</v>
       </c>
     </row>
     <row r="120">
@@ -1977,7 +1977,7 @@
         <v>0.08932403223703124</v>
       </c>
       <c r="C120" t="n">
-        <v>0.0923792707564757</v>
+        <v>0.03480189776879417</v>
       </c>
     </row>
     <row r="121">
@@ -1990,7 +1990,7 @@
         <v>0.04434459866854044</v>
       </c>
       <c r="C121" t="n">
-        <v>0.06718801710490213</v>
+        <v>0.02031277629067746</v>
       </c>
     </row>
     <row r="122">
@@ -2003,7 +2003,7 @@
         <v>0.0131319230141497</v>
       </c>
       <c r="C122" t="n">
-        <v>-0.01801466746903999</v>
+        <v>0.0006762985381678126</v>
       </c>
     </row>
     <row r="123">
@@ -2016,7 +2016,7 @@
         <v>0.04147781442639268</v>
       </c>
       <c r="C123" t="n">
-        <v>0.01638332900704023</v>
+        <v>0.0258048922722129</v>
       </c>
     </row>
     <row r="124">
@@ -2029,7 +2029,7 @@
         <v>0.03176687782497378</v>
       </c>
       <c r="C124" t="n">
-        <v>0.04138994192060443</v>
+        <v>0.0236987349281687</v>
       </c>
     </row>
     <row r="125">
@@ -2042,7 +2042,7 @@
         <v>-0.03610871940813767</v>
       </c>
       <c r="C125" t="n">
-        <v>-0.02966297052313442</v>
+        <v>-0.004259008747441018</v>
       </c>
     </row>
     <row r="126">
@@ -2055,7 +2055,7 @@
         <v>0.05356216202924662</v>
       </c>
       <c r="C126" t="n">
-        <v>0.04885876086022867</v>
+        <v>0.0289793466394201</v>
       </c>
     </row>
     <row r="127">
@@ -2068,7 +2068,7 @@
         <v>0.02081663056902152</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.02922238870197367</v>
+        <v>0.005271995540209632</v>
       </c>
     </row>
     <row r="128">
@@ -2081,7 +2081,7 @@
         <v>0.0137279502516987</v>
       </c>
       <c r="C128" t="n">
-        <v>0.05450620843456166</v>
+        <v>0.03000636847372917</v>
       </c>
     </row>
     <row r="129">
@@ -2094,7 +2094,7 @@
         <v>0.02677937050184446</v>
       </c>
       <c r="C129" t="n">
-        <v>0.02101293436414529</v>
+        <v>0.0448266518048649</v>
       </c>
     </row>
     <row r="130">
@@ -2107,7 +2107,7 @@
         <v>0.0145366796150193</v>
       </c>
       <c r="C130" t="n">
-        <v>0.01927873739525571</v>
+        <v>-0.007718462963097161</v>
       </c>
     </row>
     <row r="131">
@@ -2120,7 +2120,7 @@
         <v>-0.02341961245173092</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.04257718147709268</v>
+        <v>-0.04268207359320943</v>
       </c>
     </row>
     <row r="132">
@@ -2133,7 +2133,7 @@
         <v>0.04268246661254674</v>
       </c>
       <c r="C132" t="n">
-        <v>0.02533968154363095</v>
+        <v>0.01087110327906589</v>
       </c>
     </row>
     <row r="133">
@@ -2146,7 +2146,7 @@
         <v>-0.03202492799400349</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.04638353437801047</v>
+        <v>-0.02808343199580331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>